<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA570008867A
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -706,11 +706,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA560077165A
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -754,11 +754,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA580129846Q
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -806,11 +806,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA570032568A
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -806,11 +806,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA060105360R
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -610,11 +610,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA190071960W
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -610,11 +610,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA060220578Q
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,7 +567,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>21-09-2026 07:46:05</t>
+          <t>21-09-2026 07:46:53</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -577,17 +577,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>EA060220578Q</t>
+          <t>EA060105360R</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ARBA MARCO</t>
+          <t>ANG&amp;LY CAFFE'</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Global Starnet</t>
+          <t>NTS Networks</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -611,58 +611,6 @@
         </is>
       </c>
       <c r="J4" t="inlineStr">
-        <is>
-          <t>ELIMINA</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>21-09-2026 07:46:53</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Manuela Arigoni</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>EA060105360R</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ANG&amp;LY CAFFE'</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>NTS Networks</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>24-09-2026 06:00</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>28-09-2026 12:00</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Nessun collega</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Inviato OK</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
         <is>
           <t>ELIMINA</t>
         </is>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA910086595R
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -706,11 +706,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA230197328T
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -706,11 +706,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA900206092R
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -659,58 +659,6 @@
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>22-09-2026 11:09:51</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Riccardo Rosso</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EA900206092R</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>BAR BARAONDA DI JIN QINJING</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Snaitech Spa WG</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>28-09-2026 06:00</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>22-10-2026 12:00</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Nessun collega</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>In elaborazione</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>ELIMINA</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Allineamento Snaitech OK. Reset azione locale EA110187005R
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -514,11 +514,7 @@
           <t>Inviato OK</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>NUOVA</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🤖 [Robot] Automazione logistica e pulizia completata
</commit_message>
<xml_diff>
--- a/storico_ferie.xlsx
+++ b/storico_ferie.xlsx
@@ -1,107 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\DOC - Manuela Arigoni\SW PERSONALIZZATI\SW FERIE CLIENTI\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7F9F45-A61D-47E3-AA73-D86B169ABE6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="4125" yWindow="1365" windowWidth="21600" windowHeight="13410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>DATA_INSERIMENTO</t>
-  </si>
-  <si>
-    <t>TECNICO_INSERIMENTO</t>
-  </si>
-  <si>
-    <t>CODICE_LOCALE</t>
-  </si>
-  <si>
-    <t>NOME_LOCALE</t>
-  </si>
-  <si>
-    <t>CONCESSIONARIO</t>
-  </si>
-  <si>
-    <t>INIZIO_FERIE</t>
-  </si>
-  <si>
-    <t>FINE_FERIE</t>
-  </si>
-  <si>
-    <t>PROMEMORIA_IN_COPIA</t>
-  </si>
-  <si>
-    <t>STATO_INVIO</t>
-  </si>
-  <si>
-    <t>ROBOT_ACTION</t>
-  </si>
-  <si>
-    <t>Maurizio Adoni</t>
-  </si>
-  <si>
-    <t>TABACCHERIA BACCO</t>
-  </si>
-  <si>
-    <t>Snaitech Spa WG</t>
-  </si>
-  <si>
-    <t>Inviato OK</t>
-  </si>
-  <si>
-    <t>Nessun collega</t>
-  </si>
-  <si>
-    <t>EA110187005R</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="dd\-mm\-yyyy\ hh:mm:ss"/>
-    <numFmt numFmtId="170" formatCode="dd\-mm\-yyyy\ hh:mm"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -119,28 +49,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -428,81 +412,107 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DATA_INSERIMENTO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TECNICO_INSERIMENTO</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CODICE_LOCALE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NOME_LOCALE</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CONCESSIONARIO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>INIZIO_FERIE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>FINE_FERIE</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PROMEMORIA_IN_COPIA</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>STATO_INVIO</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ROBOT_ACTION</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <v>46288.809027777781</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4">
-        <v>46290.583333333336</v>
-      </c>
-      <c r="G2" s="4">
-        <v>46297.291666666664</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46288.80902777778</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Maurizio Adoni</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EA110187005R</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TABACCHERIA BACCO</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Snaitech Spa WG</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>46290.58333333334</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>46297.29166666666</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Nessun collega</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Inviato OK</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>